<commit_message>
rebrand: convert Rahhal codebase into Juman Girls Forum (branding, feminized copy, فصل terminology, academic stages)
</commit_message>
<xml_diff>
--- a/static/templates/participants_import_template.xlsx
+++ b/static/templates/participants_import_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المشاركون" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات التعبئة" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="المشاركات" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="تعليمات التعبئة" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -518,7 +518,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>البيئة</t>
+          <t>الفصل</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>رقم جوال المشارك</t>
+          <t>رقم جوال المشاركة</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -540,7 +540,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>عبدالله محمد الصالح</t>
+          <t>سارة عبدالله الصالح</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>البيئة الأولى</t>
+          <t>الفصل الأول</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1028,10 +1028,10 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="D3:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="قيمة غير صحيحة" error="اختر مرحلة دراسية من القائمة المتاحة فقط." type="list">
-      <formula1>"خامس ابتدائي,سادس ابتدائي,أول متوسط,ثاني متوسط,ثالث متوسط"</formula1>
+      <formula1>"أول متوسط,ثاني متوسط,ثالث متوسط,أول ثانوي,ثاني ثانوي,ثالث ثانوي"</formula1>
     </dataValidation>
     <dataValidation sqref="C3:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"البيئة الأولى,البيئة الثانية,البيئة الثالثة"</formula1>
+      <formula1>"الفصل الأول,الفصل الثاني,الفصل الثالث"</formula1>
     </dataValidation>
     <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="رقم غير صحيح" error="رقم الهوية / الإقامة يجب أن يتكون من 10 أرقام بالضبط." type="textLength" operator="equal">
       <formula1>10</formula1>
@@ -1056,7 +1056,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>قالب استيراد المشاركين — برنامج أُفق التنموي</t>
+          <t>قالب استيراد المشاركات — ملتقى جُمان للفتيات</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>1. لا تحذف أو تعدّل صف العناوين (الصف الأول) في ورقة "المشاركون".</t>
+          <t>1. لا تحذف أو تعدّل صف العناوين (الصف الأول) في ورقة "المشاركات".</t>
         </is>
       </c>
     </row>
@@ -1087,21 +1087,21 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>3. ابدأ بإدخال بيانات المشاركين الفعليين من الصف الثالث فأكثر.</t>
+          <t>3. ابدئي بإدخال بيانات المشاركات الفعليات من الصف الثالث فأكثر.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>4. لكل مشارك: عملية الاستيراد تُنشئ حساب دخول (بدون كلمة مرور — المشارك يدخل برقم</t>
+          <t>4. لكل مشاركة: عملية الاستيراد تُنشئ حساب دخول (بدون كلمة مرور — المشاركة تدخل برقم</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   الهوية فقط) وسجل بيانات المشارك مع بعض تلقائياً.</t>
+          <t xml:space="preserve">   الهوية فقط) وسجل بيانات المشاركة مع بعض تلقائياً.</t>
         </is>
       </c>
     </row>
@@ -1125,35 +1125,35 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>• رقم الهوية / الإقامة: إلزامي وفريد لكل مشارك (10 أرقام بالضبط، بدون مسافات أو رموز).</t>
+          <t>• رقم الهوية / الإقامة: إلزامي وفريد لكل مشاركة (10 أرقام بالضبط، بدون مسافات أو رموز).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>• البيئة: اسم البيئة كما هو مسجّل بالنظام بالضبط (اختر من القائمة المنسدلة).</t>
+          <t>• الفصل: اسم الفصل كما هو مسجّل بالنظام بالضبط (اختر من القائمة المنسدلة).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  إذا تُرك فارغًا، يُستورد المشارك بدون بيئة، ويمكن ربطه لاحقًا من لوحة التحكم.</t>
+          <t xml:space="preserve">  إذا تُرك فارغًا، تُستورد المشاركة بدون فصل، ويمكن ربطها لاحقًا من لوحة التحكم.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>• المرحلة الدراسية: إلزامية، اختر من القائمة المنسدلة (خامس ابتدائي إلى ثالث متوسط).</t>
+          <t>• المرحلة الدراسية: إلزامية، اختر من القائمة المنسدلة (أول متوسط إلى ثالث ثانوي).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>• رقم جوال المشارك / رقم جوال ولي الأمر: اختياريان، يفضّل تعبئتهما لأغراض التواصل والطوارئ.</t>
+          <t>• رقم جوال المشاركة / رقم جوال ولي الأمر: اختياريان، يفضّل تعبئتهما لأغراض التواصل والطوارئ.</t>
         </is>
       </c>
     </row>

</xml_diff>